<commit_message>
Clarify language background in example 90
Specify a UK customer speaking British English, and align the Mandarin explanation and audio checkpoint across CSV and Excel.
</commit_message>
<xml_diff>
--- a/T2AV评测题设计参考示例.xlsx
+++ b/T2AV评测题设计参考示例.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="100题" sheetId="3" r:id="R9f3327ae7360436f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审核规则" sheetId="4" r:id="R5f4d9b39a3784af2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="100题" sheetId="3" r:id="R90b35031bdba4641"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="审核规则" sheetId="4" r:id="Rc11f6b94b835440c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5401,7 +5401,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="B91" s="6" t="str">
-        <x:v>做10秒小餐馆里一次简短的跨语言沟通，三人同框关系清楚。外籍顾客指着菜单用英语问“Is it spicy?”，服务员听清英语却没理解，侧头看同事；同事先用中文说明顾客在问辣度，服务员再看向顾客用简短英语回答“Just a little spicy”。顾客听完点头。每人只在自己说话时开口，轮次不重叠，镜头别切到无关菜品，回答要与问题一致。 三人同框时顾客在左、服务员居中、同事在右，菜单始终由顾客手指向同一道菜。顾客提问占前两秒，服务员没理解的表情停半秒，同事用中文解释后服务员才用英语回答；三人的开口轮次不重叠，口型与两种语言各自对应。</x:v>
+        <x:v>做10秒小餐馆里一次简短的跨语言沟通，三人同框关系清楚。一位来自英国的顾客指着菜单，用自然英式英语问“Is it spicy?”，服务员听见问句但没听懂具体意思，侧头看同事；同事先用普通话说明顾客在问辣度，服务员再看向顾客用简短英语回答“Just a little spicy”。顾客听完点头。每人只在自己说话时开口，轮次不重叠，镜头别切到无关菜品，回答要与问题一致。 三人同框时顾客在左、服务员居中、同事在右，菜单始终由顾客手指向同一道菜。顾客提问占前两秒，服务员没理解的表情停半秒，同事用普通话解释后服务员才用英语回答；三人的开口轮次不重叠，口型与两种语言各自对应。</x:v>
       </x:c>
       <x:c r="C91" s="6" t="s">
         <x:v>304</x:v>
@@ -5410,7 +5410,7 @@
         <x:v>服务员听懂同事翻译后向同一位顾客回答</x:v>
       </x:c>
       <x:c r="E91" s="6" t="str">
-        <x:v>英语问答和中文解释依次清楚</x:v>
+        <x:v>英国顾客的英式英语提问、同事的普通话解释、服务员的英语回答依次清楚</x:v>
       </x:c>
       <x:c r="F91" s="6" t="str">
         <x:v>三人开口轮次不重叠，口型与各自语言对应</x:v>
@@ -5817,7 +5817,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6e80cdf666f4158"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ac565f638fd4339"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>